<commit_message>
feat(connectors): A-09 Company R anonymizer and ingest
anonymize.ts: deterministic pseudonyms from HMAC(salt, name key), salt
in data/private/r/salt (created once, 0600); one key per person across
name formats; pseudonyms avoid every real name word seen; clients
become "Client Cnn", jobs "Job Jnnn" renumbered; labels, notes and job
titles dropped; ids are salted hashes. ingest-r.ts: exports inside
data/private/r/ only -> anonymized normalized JSON in data/private/r/out/,
counts printed only; refuses payloads not stamped namesAnonymized and
any output containing a real token; file names replaced by content
hashes. Tests on synthetic samples only, including the no-surviving-
token check over the pseudonym-map keys.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/connectors/src/exports/__fixtures__/jobber-timesheets.sample.xlsx
+++ b/packages/connectors/src/exports/__fixtures__/jobber-timesheets.sample.xlsx
@@ -56,7 +56,7 @@
     <t>Avery Reed</t>
   </si>
   <si>
-    <t>Client Alpha</t>
+    <t>Brookside Dental</t>
   </si>
   <si>
     <t>Job #101 - Spring cleanup</t>
@@ -74,7 +74,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Client Beta</t>
+    <t>Maple Grove HOA</t>
   </si>
   <si>
     <t>Job #102 - Total care</t>

</xml_diff>

<commit_message>
feat(connectors): A-09 Company R anonymizer and ingest (#12)
anonymize.ts: deterministic pseudonyms from HMAC(salt, name key), salt
in data/private/r/salt (created once, 0600); one key per person across
name formats; pseudonyms avoid every real name word seen; clients
become "Client Cnn", jobs "Job Jnnn" renumbered; labels, notes and job
titles dropped; ids are salted hashes. ingest-r.ts: exports inside
data/private/r/ only -> anonymized normalized JSON in data/private/r/out/,
counts printed only; refuses payloads not stamped namesAnonymized and
any output containing a real token; file names replaced by content
hashes. Tests on synthetic samples only, including the no-surviving-
token check over the pseudonym-map keys.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/connectors/src/exports/__fixtures__/jobber-timesheets.sample.xlsx
+++ b/packages/connectors/src/exports/__fixtures__/jobber-timesheets.sample.xlsx
@@ -56,7 +56,7 @@
     <t>Avery Reed</t>
   </si>
   <si>
-    <t>Client Alpha</t>
+    <t>Brookside Dental</t>
   </si>
   <si>
     <t>Job #101 - Spring cleanup</t>
@@ -74,7 +74,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Client Beta</t>
+    <t>Maple Grove HOA</t>
   </si>
   <si>
     <t>Job #102 - Total care</t>

</xml_diff>